<commit_message>
UC3M Aerospace Engineering bölümünü ekle
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GPTxYRq3zweg2gGBU3G5XE
</commit_message>
<xml_diff>
--- a/veri/Universite_Basvuru_Tablosu.xlsx
+++ b/veri/Universite_Basvuru_Tablosu.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Üniversiteler" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Üniversiteler'!$A$1:$L$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Üniversiteler'!$A$1:$L$24</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -464,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L29"/>
+  <dimension ref="A1:L30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1513,7 +1513,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Data Science and Engineering</t>
+          <t>Aerospace Engineering (1. tercih)</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -1523,7 +1523,7 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Madrid (Leganés/Getafe)</t>
+          <t>Madrid (Leganés)</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -1545,154 +1545,204 @@
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>Early Admission: PCE/UNEDasiss yok, lise diplomasına göre değerlendirme. Yüklenecek: diploma + İng. tercüme, transkript, YKS sonucu + resmi İng. tercüme (Pazartesi tercümeye), IELTS, pasaport; SAT/AP ek başarı. Apostil gerekmez. Şartlı kabul: kayıttan önce denklik volantesi, denklik 1. yıl içinde</t>
+          <t>Tamamen İngilizce, 4 yıl / 240 ECTS, 100 kontenjan. Early Admission'da Data Science ile aynı başvuru (€150, en fazla 2 bölüm). Eksik: motivation letter (zorunlu) + €150 ödeme</t>
         </is>
       </c>
       <c r="K21" s="3" t="inlineStr"/>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>UC3M kabul ofisi maili (1 Eki 2026). Kabul sırayla – hedef gönderim 7 Eki.</t>
+          <t>Taban puan 2026/27 (1. tur, 14 üzerinden): 13,322. Kaynak: uc3m.es/bachelor-degree/aeroespace + cut-off grades.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Lund University</t>
+          <t>Universidad Carlos III de Madrid (UC3M)</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Sciences – Mathematics (B.Sc.)</t>
+          <t>Data Science and Engineering (2. tercih)</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>İsveç</t>
+          <t>İspanya</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Lund</t>
+          <t>Madrid (Leganés/Getafe)</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Ekim ortası 2026</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>15 Oca 2027</t>
-        </is>
-      </c>
+          <t>5 Eki 2026 (Early Admission)</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr"/>
       <c r="G22" s="3" t="inlineStr"/>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>71</t>
+          <t>314 (eşit)</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>95 (eşit)</t>
+          <t>801–1000</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>Türk lise matematiğinin 'Matematik 4' denkliği (belge üzerinden değerlendiriliyor)</t>
+          <t>Early Admission: PCE/UNEDasiss yok, lise diplomasına göre değerlendirme. Yüklenecek: diploma PDF (hazır), transkript, YKS + tercüme (hazır), IELTS, pasaport, motivation letter (eksik); SAT/AP ek başarı. Apostil gerekmez. Şartlı kabul: kayıttan önce denklik volantesi, denklik 1. yıl içinde</t>
         </is>
       </c>
       <c r="K22" s="3" t="inlineStr"/>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>universityadmissions.se; belgeler 1 Şub 2027'ye kadar. Kaynak: lunduniversity.lu.se</t>
+          <t>Taban puan 2026/27 (1. tur): 11,677. UC3M kabul ofisi maili (1 Eki 2026). Başvuru ücreti €150 (2 bölüme kadar); motivation letter zorunlu; dosya ≤4 MB. Hedef gönderim 7 Eki.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Università di Bologna</t>
+          <t>Lund University</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Statistical Sciences – Stats&amp;Maths</t>
+          <t>Sciences – Mathematics (B.Sc.)</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>İtalya</t>
+          <t>İsveç</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Bologna</t>
-        </is>
-      </c>
-      <c r="E23" s="3" t="inlineStr"/>
-      <c r="F23" s="3" t="inlineStr"/>
+          <t>Lund</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Ekim ortası 2026</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>15 Oca 2027</t>
+        </is>
+      </c>
       <c r="G23" s="3" t="inlineStr"/>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>123 (eşit)</t>
+          <t>71</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>130</t>
+          <t>95 (eşit)</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>İngilizce TOLC-E (€35); AB dışı kontenjan 10 kişi</t>
+          <t>Türk lise matematiğinin 'Matematik 4' denkliği (belge üzerinden değerlendiriliyor)</t>
         </is>
       </c>
       <c r="K23" s="3" t="inlineStr"/>
       <c r="L23" s="2" t="inlineStr">
         <is>
+          <t>universityadmissions.se; belgeler 1 Şub 2027'ye kadar. Kaynak: lunduniversity.lu.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Università di Bologna</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Statistical Sciences – Stats&amp;Maths</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>İtalya</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Bologna</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr"/>
+      <c r="F24" s="3" t="inlineStr"/>
+      <c r="G24" s="3" t="inlineStr"/>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>123 (eşit)</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>130</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>İngilizce TOLC-E (€35); AB dışı kontenjan 10 kişi</t>
+        </is>
+      </c>
+      <c r="K24" s="3" t="inlineStr"/>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
           <t>2027/28 başvuru çağrısı henüz yayımlanmadı.</t>
         </is>
       </c>
     </row>
-    <row r="24"/>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr">
+    <row r="25"/>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
         <is>
           <t>Açıklama</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="5" t="inlineStr">
-        <is>
-          <t>Sarı hücreler: boş bırakıldı, senin doldurman için. Sadece üniversitelerin kendi sitelerinden doğrulanan bilgiler yazıldı.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>QS 2027 ve THE 2026 (en güncel) sıraları topuniversities.com ve timeshighereducation.com üniversite sayfalarından. '(eşit)' = başka üniversiteyle aynı sırayı paylaşıyor. Tahmini kabul oranı boş.</t>
+          <t>Sarı hücreler: boş bırakıldı, senin doldurman için. Sadece üniversitelerin kendi sitelerinden doğrulanan bilgiler yazıldı.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>Ücretler 2026-27 yılına ait; 2027-28'de artabilir.</t>
+          <t>QS 2027 ve THE 2026 (en güncel) sıraları topuniversities.com ve timeshighereducation.com üniversite sayfalarından. '(eşit)' = başka üniversiteyle aynı sırayı paylaşıyor. Tahmini kabul oranı boş.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
+          <t>Ücretler 2026-27 yılına ait; 2027-28'de artabilir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
           <t>Son güncelleme: 1 Ekim 2026</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L23"/>
+  <autoFilter ref="A1:L24"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>